<commit_message>
PR_USER_CREATE と PR_PASS_RESET のテスト＆修正
</commit_message>
<xml_diff>
--- a/Docker_週報作成.xlsx
+++ b/Docker_週報作成.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ITI202302009\Documents\weeklyreport\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C48883F6-BADF-41A9-8109-D284D1C70CE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DAC2290-1DFD-477A-8815-88C491123CB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="4" xr2:uid="{949BA286-AB55-4D12-A7D1-44CDAE0F455A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="5" xr2:uid="{949BA286-AB55-4D12-A7D1-44CDAE0F455A}"/>
   </bookViews>
   <sheets>
     <sheet name="概要" sheetId="6" r:id="rId1"/>
@@ -18,25 +18,35 @@
     <sheet name="画面構成" sheetId="10" r:id="rId3"/>
     <sheet name="Docker" sheetId="11" r:id="rId4"/>
     <sheet name="python" sheetId="12" r:id="rId5"/>
-    <sheet name="Docker構成" sheetId="7" r:id="rId6"/>
-    <sheet name="練習" sheetId="8" r:id="rId7"/>
-    <sheet name="パスの指定" sheetId="1" r:id="rId8"/>
-    <sheet name="ディスク使用について" sheetId="2" r:id="rId9"/>
-    <sheet name="capter5" sheetId="3" r:id="rId10"/>
-    <sheet name="chapter6" sheetId="4" r:id="rId11"/>
-    <sheet name="Imageの出力_取込" sheetId="5" r:id="rId12"/>
+    <sheet name="MARIADB" sheetId="13" r:id="rId6"/>
+    <sheet name="パスの指定" sheetId="1" r:id="rId7"/>
+    <sheet name="ディスク使用について" sheetId="2" r:id="rId8"/>
+    <sheet name="capter5" sheetId="3" r:id="rId9"/>
+    <sheet name="chapter6" sheetId="4" r:id="rId10"/>
+    <sheet name="Imageの出力_取込" sheetId="5" r:id="rId11"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="691" uniqueCount="315">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="642" uniqueCount="278">
   <si>
     <t>Docker Image ディスク使用量とコンテンツサイズについて</t>
     <rPh sb="17" eb="20">
@@ -714,270 +724,11 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>Container1</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>【image】</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>mariaDB</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>Typescript</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>name</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>webpage</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>network</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>cmd</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>netmariadb000</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>mariadb</t>
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>【Container2】</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>【volume:bindmount】</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>file pass</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>D:\Docker\weeklyreport\web</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>D:\Docker\weeklyreport\mariadb</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>-v D:\Docker\weeklyreport\web:</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>docker create --name mariadb</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>docker create --name webpage</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>-p 3000:8080</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>--net =netmariadb000</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>docker start --name mariadb -i</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>docker image pull mariadb</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>docker image pull</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>-e MYSQL_ROOT_PASSWORD=mariadbroot</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>-e MYSQL_DATABASE=weeklyreport</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>-e MYSQL_USER=user01</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>-e MYSQL_PASSWORD=user01pass</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>-dit</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>-v D:\Docker\weeklyreport\mariadb:/var/lib/mysql</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>-p 3000:3306</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>docker network create netmariadb000</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>mariadb ログイン</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>① コンテナ起動後、コンテナ内のubuntuをbashで実行</t>
-    <rPh sb="6" eb="9">
-      <t>キドウゴ</t>
-    </rPh>
-    <rPh sb="14" eb="15">
-      <t>ナイ</t>
-    </rPh>
-    <rPh sb="28" eb="30">
-      <t>ジッコウ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>② ログイン</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>mariadb -u ユーザ名 -p</t>
-    <rPh sb="14" eb="15">
-      <t>メイ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>パスワード</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>③ mariaDBコマンド実行が可能になる</t>
-    <rPh sb="13" eb="15">
-      <t>ジッコウ</t>
-    </rPh>
-    <rPh sb="16" eb="18">
-      <t>カノウ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>④ 外部から接続する場合</t>
-    <rPh sb="2" eb="4">
-      <t>ガイブ</t>
-    </rPh>
-    <rPh sb="6" eb="8">
-      <t>セツゾク</t>
-    </rPh>
-    <rPh sb="10" eb="12">
-      <t>バアイ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>--net netmariadb000</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>docker run --name my-web -dit --net  netmariadb000 -p 8080:80 -v D:\www:/var/www/html php:8.2-apache</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>apache　PHPを利用してDB接続を行う</t>
-    <rPh sb="11" eb="13">
-      <t>リヨウ</t>
-    </rPh>
-    <rPh sb="17" eb="19">
-      <t>セツゾク</t>
-    </rPh>
-    <rPh sb="20" eb="21">
-      <t>オコナ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>① PHP apacheのイメージを取得</t>
-    <rPh sb="18" eb="20">
-      <t>シュトク</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>② DB接続の拡張機能（ドライバー）を取得</t>
-    <rPh sb="4" eb="6">
-      <t>セツゾク</t>
-    </rPh>
-    <rPh sb="7" eb="11">
-      <t>カクチョウキノウ</t>
-    </rPh>
-    <rPh sb="19" eb="21">
-      <t>シュトク</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>docker exec でコンテナ内に入り、docker-php-ext-install pdo_mysql でドライバーをインストール</t>
-    <rPh sb="17" eb="18">
-      <t>ナイ</t>
-    </rPh>
-    <rPh sb="19" eb="20">
-      <t>ハイ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>③ phpでdb接続を確認</t>
-    <rPh sb="8" eb="10">
-      <t>セツゾク</t>
-    </rPh>
-    <rPh sb="11" eb="13">
-      <t>カクニン</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>db接続のポイント</t>
-    <rPh sb="2" eb="4">
-      <t>セツゾク</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>hostはコンテナ名を指定する。</t>
-    <rPh sb="9" eb="10">
-      <t>メイ</t>
-    </rPh>
-    <rPh sb="11" eb="13">
-      <t>シテイ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>dbコンテナとapacheコンテナを同じnetで作成する。</t>
-    <rPh sb="18" eb="19">
-      <t>オナ</t>
-    </rPh>
-    <rPh sb="24" eb="26">
-      <t>サクセイ</t>
-    </rPh>
     <phoneticPr fontId="1"/>
   </si>
   <si>
@@ -2033,10 +1784,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>docker exec -it dbコンテナ名 bash</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>作成</t>
     <rPh sb="0" eb="2">
       <t>サクセイ</t>
@@ -2252,6 +1999,46 @@
     <rPh sb="17" eb="19">
       <t>キドウ</t>
     </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>DATETIME</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>PROC_NAME</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ERR_CODE</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ERR_MESSAGE</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ERR_PARAM</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>INT(11)</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>VARCHAR(30)</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ID</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>CURRENT_TIMESTAMP()</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>AUTO_INCREMENT</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -2324,7 +2111,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2345,12 +2132,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="5" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -2362,92 +2143,12 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="1">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -2459,7 +2160,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -2484,52 +2185,16 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="1" applyFill="1">
@@ -4027,368 +3692,6 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>19050</xdr:colOff>
-      <xdr:row>31</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>28</xdr:col>
-      <xdr:colOff>263529</xdr:colOff>
-      <xdr:row>32</xdr:row>
-      <xdr:rowOff>131484</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="図 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{72ABFC51-7EC3-7926-F24F-567675DCC336}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="5810250" y="5953125"/>
-          <a:ext cx="4587879" cy="281979"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>38</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>39</xdr:col>
-      <xdr:colOff>206930</xdr:colOff>
-      <xdr:row>50</xdr:row>
-      <xdr:rowOff>15560</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="図 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8C33B864-2752-C31D-EC02-06AB1685086C}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="5791200" y="7239000"/>
-          <a:ext cx="8526065" cy="2295845"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>53</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>29</xdr:col>
-      <xdr:colOff>19709</xdr:colOff>
-      <xdr:row>60</xdr:row>
-      <xdr:rowOff>114502</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="図 3">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6120C943-632D-0FA4-8149-7E96616AF7D4}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="5791200" y="10096500"/>
-          <a:ext cx="4725059" cy="1448002"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>63</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>41</xdr:col>
-      <xdr:colOff>267987</xdr:colOff>
-      <xdr:row>76</xdr:row>
-      <xdr:rowOff>53694</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="図 4">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B3C3C4B3-3C92-2841-E7DC-ABFF06655CC6}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="5730240" y="12001500"/>
-          <a:ext cx="9221487" cy="2534004"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>79</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>30</xdr:col>
-      <xdr:colOff>160742</xdr:colOff>
-      <xdr:row>96</xdr:row>
-      <xdr:rowOff>88094</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="図 5">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9FF3C702-B84F-7D80-3BB6-1E7719C85778}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="5730240" y="15049500"/>
-          <a:ext cx="5172797" cy="3324689"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>85725</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>1117</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>65058</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="図 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8DB17855-C141-4DDB-8249-5302DF7A2ED9}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="1228725"/>
-          <a:ext cx="8002117" cy="2076738"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>1905</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>416279</xdr:colOff>
-      <xdr:row>51</xdr:row>
-      <xdr:rowOff>103521</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="図 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AA98C907-C190-4068-BCBC-565B0A1A41A4}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="5145405"/>
-          <a:ext cx="7083779" cy="4673616"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>52</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>191271</xdr:colOff>
-      <xdr:row>65</xdr:row>
-      <xdr:rowOff>72744</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="図 3">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AEBE43F2-7DA6-4643-9313-02B550F08003}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="9925050"/>
-          <a:ext cx="5525271" cy="2530194"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>0</xdr:row>
@@ -4434,7 +3737,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -4571,7 +3874,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -4620,7 +3923,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -4890,7 +4193,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -5389,7 +4692,7 @@
         <v>78</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>172</v>
+        <v>126</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -5397,7 +4700,7 @@
         <v>82</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>170</v>
+        <v>124</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -5405,7 +4708,7 @@
         <v>76</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>171</v>
+        <v>125</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -5413,7 +4716,7 @@
         <v>77</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>173</v>
+        <v>127</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -5433,93 +4736,93 @@
     </row>
     <row r="13" spans="1:8">
       <c r="A13" s="1" t="s">
-        <v>132</v>
+        <v>86</v>
       </c>
     </row>
     <row r="14" spans="1:8">
       <c r="A14" s="1" t="s">
-        <v>133</v>
+        <v>87</v>
       </c>
     </row>
     <row r="16" spans="1:8">
       <c r="A16" s="1" t="s">
-        <v>134</v>
+        <v>88</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>138</v>
+        <v>92</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>139</v>
+        <v>93</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>143</v>
+        <v>97</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>144</v>
+        <v>98</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="1" t="s">
-        <v>135</v>
+        <v>89</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>140</v>
+        <v>94</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" s="1" t="s">
-        <v>136</v>
+        <v>90</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>141</v>
+        <v>95</v>
       </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" s="1" t="s">
-        <v>137</v>
+        <v>91</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>142</v>
+        <v>96</v>
       </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" s="1" t="s">
-        <v>146</v>
+        <v>100</v>
       </c>
     </row>
     <row r="22" spans="1:6">
       <c r="A22" s="1" t="s">
-        <v>145</v>
+        <v>99</v>
       </c>
     </row>
     <row r="24" spans="1:6">
       <c r="A24" s="1" t="s">
-        <v>147</v>
+        <v>101</v>
       </c>
     </row>
     <row r="25" spans="1:6">
       <c r="A25" s="1" t="s">
-        <v>148</v>
+        <v>102</v>
       </c>
     </row>
     <row r="26" spans="1:6">
       <c r="A26" s="1" t="s">
-        <v>149</v>
+        <v>103</v>
       </c>
     </row>
     <row r="27" spans="1:6">
       <c r="A27" s="1" t="s">
-        <v>150</v>
+        <v>104</v>
       </c>
     </row>
     <row r="30" spans="1:6">
       <c r="A30" s="1" t="s">
-        <v>151</v>
+        <v>105</v>
       </c>
     </row>
     <row r="31" spans="1:6">
       <c r="A31" s="1" t="s">
-        <v>152</v>
+        <v>106</v>
       </c>
     </row>
   </sheetData>
@@ -5529,211 +4832,6 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E00EB3AB-A229-45B6-BAF0-CBFC690801AC}">
-  <dimension ref="A1:A72"/>
-  <sheetFormatPr defaultColWidth="8.75" defaultRowHeight="15.75"/>
-  <cols>
-    <col min="1" max="16384" width="8.75" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:1" s="6" customFormat="1">
-      <c r="A1" s="6" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" s="7" customFormat="1">
-      <c r="A2" s="7" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1">
-      <c r="A3" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1">
-      <c r="A5" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1">
-      <c r="A7" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1">
-      <c r="A8" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1">
-      <c r="A10" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1">
-      <c r="A11" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1">
-      <c r="A13" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1">
-      <c r="A14" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1">
-      <c r="A16" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1">
-      <c r="A17" s="1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" s="7" customFormat="1">
-      <c r="A22" s="7" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1">
-      <c r="A23" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="37" spans="1:1" s="7" customFormat="1">
-      <c r="A37" s="7" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="38" spans="1:1">
-      <c r="A38" s="1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="40" spans="1:1">
-      <c r="A40" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="41" spans="1:1">
-      <c r="A41" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="43" spans="1:1">
-      <c r="A43" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="44" spans="1:1">
-      <c r="A44" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="45" spans="1:1">
-      <c r="A45" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="47" spans="1:1">
-      <c r="A47" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="48" spans="1:1">
-      <c r="A48" s="1" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="50" spans="1:1">
-      <c r="A50" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="51" spans="1:1">
-      <c r="A51" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="54" spans="1:1">
-      <c r="A54" s="1" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="55" spans="1:1">
-      <c r="A55" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="56" spans="1:1">
-      <c r="A56" s="1" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="57" spans="1:1">
-      <c r="A57" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="60" spans="1:1" s="7" customFormat="1">
-      <c r="A60" s="7" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="62" spans="1:1">
-      <c r="A62" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="63" spans="1:1">
-      <c r="A63" s="1" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="65" spans="1:1">
-      <c r="A65" s="1" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="66" spans="1:1">
-      <c r="A66" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="68" spans="1:1">
-      <c r="A68" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="69" spans="1:1">
-      <c r="A69" s="1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="71" spans="1:1">
-      <c r="A71" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="72" spans="1:1">
-      <c r="A72" s="1" t="s">
-        <v>42</v>
-      </c>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="1"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{951AFAFC-64BB-48A0-B0C5-F9BF0356E726}">
   <dimension ref="A1:C101"/>
   <sheetFormatPr defaultColWidth="8.75" defaultRowHeight="15.75"/>
@@ -5862,7 +4960,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A15534C-900B-4E1C-9ED3-A15604A7DB2E}">
   <dimension ref="A1:A29"/>
   <sheetFormatPr defaultColWidth="8.75" defaultRowHeight="15.75"/>
@@ -5919,7 +5017,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7AB8AA92-C104-4402-9D79-D3850C7E3800}">
-  <dimension ref="A1:I136"/>
+  <dimension ref="A1:I138"/>
   <sheetFormatPr defaultColWidth="4.75" defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="1" width="4.75" style="1"/>
@@ -5933,1517 +5031,1561 @@
     <col min="9" max="16384" width="4.75" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="23" customFormat="1">
-      <c r="A1" s="23" t="s">
-        <v>305</v>
+    <row r="1" spans="1:9" s="11" customFormat="1">
+      <c r="A1" s="11" t="s">
+        <v>258</v>
       </c>
     </row>
     <row r="2" spans="1:9">
       <c r="A2" s="1" t="s">
-        <v>306</v>
+        <v>259</v>
       </c>
     </row>
     <row r="3" spans="1:9">
       <c r="A3" s="1" t="s">
-        <v>307</v>
+        <v>260</v>
       </c>
     </row>
     <row r="5" spans="1:9">
       <c r="I5" s="1" t="s">
-        <v>279</v>
+        <v>232</v>
       </c>
     </row>
     <row r="6" spans="1:9">
       <c r="B6" s="1">
         <v>1</v>
       </c>
-      <c r="C6" s="21" t="s">
-        <v>182</v>
-      </c>
-      <c r="D6" s="21" t="s">
-        <v>185</v>
-      </c>
-      <c r="E6" s="21"/>
-      <c r="F6" s="21"/>
-      <c r="G6" s="21"/>
-      <c r="H6" s="21"/>
+      <c r="C6" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
+      <c r="G6" s="9"/>
+      <c r="H6" s="9"/>
       <c r="I6" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
     </row>
     <row r="7" spans="1:9">
       <c r="C7" s="7" t="s">
-        <v>162</v>
+        <v>116</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>163</v>
+        <v>117</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>164</v>
+        <v>118</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>166</v>
+        <v>120</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>188</v>
+        <v>142</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>167</v>
+        <v>121</v>
       </c>
     </row>
     <row r="8" spans="1:9">
       <c r="C8" s="1" t="s">
-        <v>180</v>
+        <v>134</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>181</v>
+        <v>135</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>185</v>
+        <v>139</v>
       </c>
     </row>
     <row r="9" spans="1:9">
       <c r="C9" s="1" t="s">
-        <v>183</v>
+        <v>137</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>159</v>
+        <v>113</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>215</v>
+        <v>169</v>
       </c>
     </row>
     <row r="10" spans="1:9">
       <c r="C10" s="1" t="s">
-        <v>256</v>
+        <v>210</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>228</v>
+        <v>268</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
     </row>
     <row r="11" spans="1:9">
       <c r="C11" s="1" t="s">
-        <v>302</v>
+        <v>255</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>159</v>
+        <v>113</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
     </row>
     <row r="12" spans="1:9">
       <c r="C12" s="1" t="s">
-        <v>303</v>
+        <v>256</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>228</v>
+        <v>268</v>
       </c>
     </row>
     <row r="13" spans="1:9">
       <c r="C13" s="1" t="s">
-        <v>304</v>
+        <v>257</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>159</v>
+        <v>113</v>
       </c>
     </row>
     <row r="15" spans="1:9">
       <c r="B15" s="1">
         <v>2</v>
       </c>
-      <c r="C15" s="21" t="s">
-        <v>153</v>
-      </c>
-      <c r="D15" s="21" t="s">
-        <v>186</v>
-      </c>
-      <c r="E15" s="21"/>
-      <c r="F15" s="21"/>
-      <c r="G15" s="21"/>
-      <c r="H15" s="21"/>
+      <c r="C15" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="E15" s="9"/>
+      <c r="F15" s="9"/>
+      <c r="G15" s="9"/>
+      <c r="H15" s="9"/>
       <c r="I15" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
     </row>
     <row r="16" spans="1:9">
       <c r="C16" s="7" t="s">
-        <v>162</v>
+        <v>116</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>163</v>
+        <v>117</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>164</v>
+        <v>118</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>166</v>
+        <v>120</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>188</v>
+        <v>142</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>167</v>
+        <v>121</v>
       </c>
     </row>
     <row r="17" spans="2:8">
       <c r="C17" s="1" t="s">
-        <v>175</v>
+        <v>129</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>159</v>
+        <v>113</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>219</v>
+        <v>173</v>
       </c>
     </row>
     <row r="18" spans="2:8">
       <c r="C18" s="1" t="s">
-        <v>154</v>
+        <v>108</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>160</v>
+        <v>114</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>216</v>
+        <v>170</v>
       </c>
     </row>
     <row r="19" spans="2:8">
       <c r="C19" s="1" t="s">
-        <v>155</v>
+        <v>109</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>160</v>
+        <v>114</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>217</v>
+        <v>171</v>
       </c>
     </row>
     <row r="20" spans="2:8">
       <c r="C20" s="1" t="s">
-        <v>156</v>
+        <v>110</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>160</v>
+        <v>114</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>218</v>
+        <v>172</v>
       </c>
     </row>
     <row r="21" spans="2:8">
       <c r="C21" s="1" t="s">
-        <v>157</v>
+        <v>111</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>161</v>
+        <v>115</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>169</v>
+        <v>123</v>
       </c>
     </row>
     <row r="22" spans="2:8">
       <c r="C22" s="1" t="s">
-        <v>158</v>
+        <v>112</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>161</v>
+        <v>115</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>168</v>
+        <v>122</v>
       </c>
     </row>
     <row r="23" spans="2:8">
       <c r="C23" s="1" t="s">
-        <v>180</v>
+        <v>134</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>181</v>
+        <v>135</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>185</v>
+        <v>139</v>
       </c>
     </row>
     <row r="24" spans="2:8">
       <c r="C24" s="1" t="s">
-        <v>256</v>
+        <v>210</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>228</v>
+        <v>268</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
     </row>
     <row r="25" spans="2:8">
       <c r="C25" s="1" t="s">
-        <v>302</v>
+        <v>255</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>159</v>
+        <v>113</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
     </row>
     <row r="26" spans="2:8">
       <c r="C26" s="1" t="s">
-        <v>303</v>
+        <v>256</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>228</v>
+        <v>268</v>
       </c>
     </row>
     <row r="27" spans="2:8">
       <c r="C27" s="1" t="s">
-        <v>304</v>
+        <v>257</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>159</v>
+        <v>113</v>
       </c>
     </row>
     <row r="29" spans="2:8">
       <c r="B29" s="1">
         <v>3</v>
       </c>
-      <c r="C29" s="21" t="s">
-        <v>184</v>
-      </c>
-      <c r="D29" s="21" t="s">
-        <v>119</v>
-      </c>
-      <c r="E29" s="21"/>
-      <c r="F29" s="21"/>
-      <c r="G29" s="21"/>
-      <c r="H29" s="21"/>
+      <c r="C29" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="D29" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="E29" s="9"/>
+      <c r="F29" s="9"/>
+      <c r="G29" s="9"/>
+      <c r="H29" s="9"/>
     </row>
     <row r="30" spans="2:8">
       <c r="C30" s="7" t="s">
-        <v>162</v>
+        <v>116</v>
       </c>
       <c r="D30" s="7" t="s">
-        <v>163</v>
+        <v>117</v>
       </c>
       <c r="E30" s="7" t="s">
-        <v>164</v>
+        <v>118</v>
       </c>
       <c r="F30" s="7" t="s">
-        <v>166</v>
+        <v>120</v>
       </c>
       <c r="G30" s="7" t="s">
-        <v>188</v>
+        <v>142</v>
       </c>
       <c r="H30" s="7" t="s">
-        <v>167</v>
+        <v>121</v>
       </c>
     </row>
     <row r="31" spans="2:8">
       <c r="C31" s="1" t="s">
-        <v>175</v>
+        <v>129</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>159</v>
+        <v>113</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>219</v>
+        <v>173</v>
       </c>
     </row>
     <row r="32" spans="2:8">
       <c r="C32" s="1" t="s">
-        <v>184</v>
+        <v>138</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>276</v>
+        <v>230</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
       <c r="H32" s="1" t="s">
-        <v>119</v>
+        <v>85</v>
       </c>
     </row>
     <row r="33" spans="2:8">
       <c r="C33" s="1" t="s">
-        <v>189</v>
+        <v>143</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>191</v>
+        <v>145</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>212</v>
+        <v>166</v>
       </c>
     </row>
     <row r="34" spans="2:8">
       <c r="C34" s="1" t="s">
-        <v>190</v>
+        <v>144</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>191</v>
+        <v>145</v>
       </c>
       <c r="H34" s="1" t="s">
-        <v>213</v>
+        <v>167</v>
       </c>
     </row>
     <row r="35" spans="2:8">
       <c r="C35" s="1" t="s">
-        <v>256</v>
+        <v>210</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>228</v>
+        <v>268</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
     </row>
     <row r="36" spans="2:8">
       <c r="C36" s="1" t="s">
-        <v>302</v>
+        <v>255</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>159</v>
+        <v>113</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
     </row>
     <row r="37" spans="2:8">
       <c r="C37" s="1" t="s">
-        <v>303</v>
+        <v>256</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>228</v>
+        <v>268</v>
       </c>
     </row>
     <row r="38" spans="2:8">
       <c r="C38" s="1" t="s">
-        <v>304</v>
+        <v>257</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>159</v>
+        <v>113</v>
       </c>
     </row>
     <row r="41" spans="2:8">
       <c r="B41" s="1">
         <v>4</v>
       </c>
-      <c r="C41" s="21" t="s">
-        <v>261</v>
-      </c>
-      <c r="D41" s="21" t="s">
-        <v>262</v>
-      </c>
-      <c r="E41" s="21"/>
-      <c r="F41" s="21"/>
-      <c r="G41" s="21"/>
-      <c r="H41" s="21"/>
+      <c r="C41" s="9" t="s">
+        <v>215</v>
+      </c>
+      <c r="D41" s="9" t="s">
+        <v>216</v>
+      </c>
+      <c r="E41" s="9"/>
+      <c r="F41" s="9"/>
+      <c r="G41" s="9"/>
+      <c r="H41" s="9"/>
     </row>
     <row r="42" spans="2:8">
       <c r="C42" s="7" t="s">
-        <v>162</v>
+        <v>116</v>
       </c>
       <c r="D42" s="7" t="s">
-        <v>163</v>
+        <v>117</v>
       </c>
       <c r="E42" s="7" t="s">
-        <v>164</v>
+        <v>118</v>
       </c>
       <c r="F42" s="7" t="s">
-        <v>166</v>
+        <v>120</v>
       </c>
       <c r="G42" s="7" t="s">
-        <v>188</v>
+        <v>142</v>
       </c>
       <c r="H42" s="7" t="s">
-        <v>167</v>
+        <v>121</v>
       </c>
     </row>
     <row r="43" spans="2:8">
       <c r="C43" s="1" t="s">
-        <v>175</v>
+        <v>129</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>159</v>
+        <v>113</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
       <c r="H43" s="1" t="s">
-        <v>219</v>
+        <v>173</v>
       </c>
     </row>
     <row r="44" spans="2:8">
       <c r="C44" s="1" t="s">
-        <v>281</v>
+        <v>234</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>159</v>
+        <v>113</v>
       </c>
       <c r="E44" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="H44" s="1" t="s">
         <v>165</v>
-      </c>
-      <c r="H44" s="1" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="45" spans="2:8">
       <c r="C45" s="1" t="s">
-        <v>194</v>
+        <v>148</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>161</v>
+        <v>115</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
       <c r="H45" s="1" t="s">
-        <v>265</v>
+        <v>219</v>
       </c>
     </row>
     <row r="46" spans="2:8">
       <c r="C46" s="1" t="s">
-        <v>261</v>
+        <v>215</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>160</v>
+        <v>114</v>
       </c>
       <c r="H46" s="1" t="s">
-        <v>262</v>
+        <v>216</v>
       </c>
     </row>
     <row r="47" spans="2:8">
       <c r="C47" s="1" t="s">
-        <v>256</v>
+        <v>210</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>228</v>
+        <v>268</v>
       </c>
       <c r="G47" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
     </row>
     <row r="48" spans="2:8">
       <c r="C48" s="1" t="s">
-        <v>302</v>
+        <v>255</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>159</v>
+        <v>113</v>
       </c>
       <c r="G48" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
     </row>
     <row r="49" spans="2:8">
       <c r="C49" s="1" t="s">
-        <v>303</v>
+        <v>256</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>228</v>
+        <v>268</v>
       </c>
     </row>
     <row r="50" spans="2:8">
       <c r="C50" s="1" t="s">
-        <v>304</v>
+        <v>257</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>159</v>
+        <v>113</v>
       </c>
     </row>
     <row r="52" spans="2:8">
       <c r="B52" s="1">
         <v>5</v>
       </c>
-      <c r="C52" s="21" t="s">
-        <v>270</v>
-      </c>
-      <c r="D52" s="21" t="s">
-        <v>268</v>
-      </c>
-      <c r="E52" s="21"/>
-      <c r="F52" s="21"/>
-      <c r="G52" s="21"/>
-      <c r="H52" s="21"/>
+      <c r="C52" s="9" t="s">
+        <v>224</v>
+      </c>
+      <c r="D52" s="9" t="s">
+        <v>222</v>
+      </c>
+      <c r="E52" s="9"/>
+      <c r="F52" s="9"/>
+      <c r="G52" s="9"/>
+      <c r="H52" s="9"/>
     </row>
     <row r="53" spans="2:8">
       <c r="C53" s="7" t="s">
-        <v>162</v>
+        <v>116</v>
       </c>
       <c r="D53" s="7" t="s">
-        <v>163</v>
+        <v>117</v>
       </c>
       <c r="E53" s="7" t="s">
-        <v>164</v>
+        <v>118</v>
       </c>
       <c r="F53" s="7" t="s">
-        <v>166</v>
+        <v>120</v>
       </c>
       <c r="G53" s="7" t="s">
-        <v>188</v>
+        <v>142</v>
       </c>
       <c r="H53" s="7" t="s">
-        <v>167</v>
+        <v>121</v>
       </c>
     </row>
     <row r="54" spans="2:8">
       <c r="C54" s="1" t="s">
-        <v>175</v>
+        <v>129</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>159</v>
+        <v>113</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
       <c r="H54" s="1" t="s">
-        <v>219</v>
+        <v>173</v>
       </c>
     </row>
     <row r="55" spans="2:8">
       <c r="C55" s="1" t="s">
-        <v>281</v>
+        <v>234</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>159</v>
+        <v>113</v>
       </c>
       <c r="E55" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="H55" s="1" t="s">
         <v>165</v>
-      </c>
-      <c r="H55" s="1" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="56" spans="2:8">
       <c r="C56" s="1" t="s">
-        <v>194</v>
+        <v>148</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>161</v>
+        <v>115</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
       <c r="H56" s="1" t="s">
-        <v>265</v>
+        <v>219</v>
       </c>
     </row>
     <row r="57" spans="2:8">
       <c r="C57" s="1" t="s">
-        <v>200</v>
+        <v>154</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>201</v>
+        <v>155</v>
       </c>
       <c r="H57" s="1" t="s">
-        <v>220</v>
+        <v>174</v>
       </c>
     </row>
     <row r="58" spans="2:8">
       <c r="C58" s="1" t="s">
-        <v>266</v>
+        <v>220</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>201</v>
+        <v>155</v>
       </c>
       <c r="H58" s="1" t="s">
-        <v>209</v>
+        <v>163</v>
       </c>
     </row>
     <row r="59" spans="2:8">
       <c r="C59" s="1" t="s">
-        <v>267</v>
+        <v>221</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>201</v>
+        <v>155</v>
       </c>
       <c r="H59" s="1" t="s">
-        <v>221</v>
+        <v>175</v>
       </c>
     </row>
     <row r="60" spans="2:8">
       <c r="C60" s="1" t="s">
-        <v>256</v>
+        <v>210</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>228</v>
+        <v>268</v>
       </c>
       <c r="G60" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
     </row>
     <row r="61" spans="2:8">
       <c r="C61" s="1" t="s">
-        <v>302</v>
+        <v>255</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>159</v>
+        <v>113</v>
       </c>
       <c r="G61" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
     </row>
     <row r="62" spans="2:8">
       <c r="C62" s="1" t="s">
-        <v>303</v>
+        <v>256</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>228</v>
+        <v>268</v>
       </c>
     </row>
     <row r="63" spans="2:8">
       <c r="C63" s="1" t="s">
-        <v>304</v>
+        <v>257</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>159</v>
+        <v>113</v>
       </c>
     </row>
     <row r="65" spans="2:8">
       <c r="B65" s="1">
         <v>6</v>
       </c>
-      <c r="C65" s="21" t="s">
-        <v>205</v>
-      </c>
-      <c r="D65" s="21" t="s">
-        <v>204</v>
-      </c>
-      <c r="E65" s="21"/>
-      <c r="F65" s="21"/>
-      <c r="G65" s="21"/>
-      <c r="H65" s="21"/>
+      <c r="C65" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="D65" s="9" t="s">
+        <v>158</v>
+      </c>
+      <c r="E65" s="9"/>
+      <c r="F65" s="9"/>
+      <c r="G65" s="9"/>
+      <c r="H65" s="9"/>
     </row>
     <row r="66" spans="2:8">
       <c r="C66" s="7" t="s">
-        <v>162</v>
+        <v>116</v>
       </c>
       <c r="D66" s="7" t="s">
-        <v>163</v>
+        <v>117</v>
       </c>
       <c r="E66" s="7" t="s">
-        <v>164</v>
+        <v>118</v>
       </c>
       <c r="F66" s="7" t="s">
-        <v>166</v>
+        <v>120</v>
       </c>
       <c r="G66" s="7" t="s">
-        <v>188</v>
+        <v>142</v>
       </c>
       <c r="H66" s="7" t="s">
-        <v>167</v>
+        <v>121</v>
       </c>
     </row>
     <row r="67" spans="2:8">
       <c r="C67" s="1" t="s">
-        <v>175</v>
+        <v>129</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>159</v>
+        <v>113</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
       <c r="F67" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
       <c r="H67" s="1" t="s">
-        <v>219</v>
+        <v>173</v>
       </c>
     </row>
     <row r="68" spans="2:8">
       <c r="C68" s="1" t="s">
-        <v>281</v>
+        <v>234</v>
       </c>
       <c r="D68" s="1" t="s">
-        <v>159</v>
+        <v>113</v>
       </c>
       <c r="E68" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="H68" s="1" t="s">
         <v>165</v>
-      </c>
-      <c r="H68" s="1" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="69" spans="2:8">
       <c r="C69" s="1" t="s">
-        <v>194</v>
+        <v>148</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>161</v>
+        <v>115</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
       <c r="H69" s="1" t="s">
-        <v>265</v>
+        <v>219</v>
       </c>
     </row>
     <row r="70" spans="2:8">
       <c r="C70" s="1" t="s">
-        <v>263</v>
+        <v>217</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>206</v>
+        <v>160</v>
       </c>
       <c r="H70" s="1" t="s">
-        <v>222</v>
+        <v>176</v>
       </c>
     </row>
     <row r="71" spans="2:8">
       <c r="C71" s="1" t="s">
-        <v>264</v>
+        <v>218</v>
       </c>
       <c r="D71" s="1" t="s">
-        <v>206</v>
+        <v>160</v>
       </c>
       <c r="H71" s="1" t="s">
-        <v>223</v>
+        <v>177</v>
       </c>
     </row>
     <row r="72" spans="2:8">
       <c r="C72" s="1" t="s">
-        <v>256</v>
+        <v>210</v>
       </c>
       <c r="D72" s="1" t="s">
-        <v>228</v>
+        <v>268</v>
       </c>
       <c r="G72" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
     </row>
     <row r="73" spans="2:8">
       <c r="C73" s="1" t="s">
-        <v>302</v>
+        <v>255</v>
       </c>
       <c r="D73" s="1" t="s">
-        <v>159</v>
+        <v>113</v>
       </c>
       <c r="G73" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
     </row>
     <row r="74" spans="2:8">
       <c r="C74" s="1" t="s">
-        <v>303</v>
+        <v>256</v>
       </c>
       <c r="D74" s="1" t="s">
-        <v>228</v>
+        <v>268</v>
       </c>
     </row>
     <row r="75" spans="2:8">
       <c r="C75" s="1" t="s">
-        <v>304</v>
+        <v>257</v>
       </c>
       <c r="D75" s="1" t="s">
-        <v>159</v>
+        <v>113</v>
       </c>
     </row>
     <row r="77" spans="2:8">
       <c r="B77" s="1">
         <v>7</v>
       </c>
-      <c r="C77" s="21" t="s">
-        <v>174</v>
-      </c>
-      <c r="D77" s="21" t="s">
-        <v>187</v>
-      </c>
-      <c r="E77" s="21"/>
-      <c r="F77" s="21"/>
-      <c r="G77" s="21"/>
-      <c r="H77" s="21"/>
+      <c r="C77" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="D77" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="E77" s="9"/>
+      <c r="F77" s="9"/>
+      <c r="G77" s="9"/>
+      <c r="H77" s="9"/>
     </row>
     <row r="78" spans="2:8">
       <c r="C78" s="7" t="s">
-        <v>162</v>
+        <v>116</v>
       </c>
       <c r="D78" s="7" t="s">
-        <v>163</v>
+        <v>117</v>
       </c>
       <c r="E78" s="7" t="s">
-        <v>164</v>
+        <v>118</v>
       </c>
       <c r="F78" s="7" t="s">
-        <v>166</v>
+        <v>120</v>
       </c>
       <c r="G78" s="7" t="s">
-        <v>188</v>
+        <v>142</v>
       </c>
       <c r="H78" s="7" t="s">
-        <v>167</v>
+        <v>121</v>
       </c>
     </row>
     <row r="79" spans="2:8">
       <c r="C79" s="1" t="s">
-        <v>175</v>
+        <v>129</v>
       </c>
       <c r="D79" s="1" t="s">
-        <v>159</v>
+        <v>113</v>
       </c>
       <c r="E79" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
       <c r="F79" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
       <c r="H79" s="1" t="s">
-        <v>219</v>
+        <v>173</v>
       </c>
     </row>
     <row r="80" spans="2:8">
       <c r="C80" s="1" t="s">
-        <v>281</v>
+        <v>234</v>
       </c>
       <c r="D80" s="1" t="s">
-        <v>159</v>
+        <v>113</v>
       </c>
       <c r="E80" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="H80" s="1" t="s">
         <v>165</v>
-      </c>
-      <c r="H80" s="1" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="81" spans="2:8">
       <c r="C81" s="1" t="s">
-        <v>176</v>
+        <v>130</v>
       </c>
       <c r="D81" s="1" t="s">
-        <v>161</v>
+        <v>115</v>
       </c>
       <c r="E81" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
       <c r="G81" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
       <c r="H81" s="1" t="s">
-        <v>177</v>
+        <v>131</v>
       </c>
     </row>
     <row r="82" spans="2:8">
       <c r="C82" s="1" t="s">
-        <v>178</v>
+        <v>132</v>
       </c>
       <c r="D82" s="1" t="s">
-        <v>192</v>
+        <v>146</v>
       </c>
       <c r="G82" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
       <c r="H82" s="1" t="s">
-        <v>143</v>
+        <v>97</v>
       </c>
     </row>
     <row r="83" spans="2:8">
       <c r="C83" s="1" t="s">
-        <v>179</v>
+        <v>133</v>
       </c>
       <c r="D83" s="1" t="s">
-        <v>192</v>
+        <v>146</v>
       </c>
       <c r="H83" s="1" t="s">
-        <v>214</v>
+        <v>168</v>
       </c>
     </row>
     <row r="84" spans="2:8">
       <c r="C84" s="1" t="s">
-        <v>256</v>
+        <v>210</v>
       </c>
       <c r="D84" s="1" t="s">
-        <v>228</v>
+        <v>268</v>
       </c>
       <c r="G84" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
     </row>
     <row r="85" spans="2:8">
       <c r="C85" s="1" t="s">
-        <v>302</v>
+        <v>255</v>
       </c>
       <c r="D85" s="1" t="s">
-        <v>159</v>
+        <v>113</v>
       </c>
       <c r="G85" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
     </row>
     <row r="86" spans="2:8">
       <c r="C86" s="1" t="s">
-        <v>303</v>
+        <v>256</v>
       </c>
       <c r="D86" s="1" t="s">
-        <v>228</v>
+        <v>268</v>
       </c>
     </row>
     <row r="87" spans="2:8">
       <c r="C87" s="1" t="s">
-        <v>304</v>
+        <v>257</v>
       </c>
       <c r="D87" s="1" t="s">
-        <v>159</v>
+        <v>113</v>
       </c>
     </row>
     <row r="89" spans="2:8">
       <c r="B89" s="1">
         <v>8</v>
       </c>
-      <c r="C89" s="21" t="s">
-        <v>277</v>
-      </c>
-      <c r="D89" s="21" t="s">
-        <v>233</v>
-      </c>
-      <c r="E89" s="21"/>
-      <c r="F89" s="21"/>
-      <c r="G89" s="21"/>
-      <c r="H89" s="21"/>
+      <c r="C89" s="9" t="s">
+        <v>231</v>
+      </c>
+      <c r="D89" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="E89" s="9"/>
+      <c r="F89" s="9"/>
+      <c r="G89" s="9"/>
+      <c r="H89" s="9"/>
     </row>
     <row r="90" spans="2:8">
       <c r="C90" s="7" t="s">
-        <v>162</v>
+        <v>116</v>
       </c>
       <c r="D90" s="7" t="s">
-        <v>163</v>
+        <v>117</v>
       </c>
       <c r="E90" s="7" t="s">
-        <v>164</v>
+        <v>118</v>
       </c>
       <c r="F90" s="7" t="s">
-        <v>166</v>
+        <v>120</v>
       </c>
       <c r="G90" s="7" t="s">
-        <v>188</v>
+        <v>142</v>
       </c>
       <c r="H90" s="7" t="s">
-        <v>167</v>
+        <v>121</v>
       </c>
     </row>
     <row r="91" spans="2:8">
       <c r="C91" s="1" t="s">
-        <v>236</v>
+        <v>190</v>
       </c>
       <c r="D91" s="1" t="s">
-        <v>159</v>
+        <v>113</v>
       </c>
       <c r="E91" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
       <c r="F91" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
       <c r="H91" s="1" t="s">
-        <v>237</v>
+        <v>191</v>
       </c>
     </row>
     <row r="92" spans="2:8">
       <c r="C92" s="1" t="s">
-        <v>256</v>
+        <v>210</v>
       </c>
       <c r="D92" s="1" t="s">
-        <v>228</v>
+        <v>268</v>
       </c>
       <c r="E92" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
       <c r="H92" s="1" t="s">
-        <v>257</v>
+        <v>211</v>
       </c>
     </row>
     <row r="93" spans="2:8">
       <c r="C93" s="1" t="s">
-        <v>280</v>
+        <v>233</v>
       </c>
       <c r="D93" s="1" t="s">
-        <v>159</v>
+        <v>113</v>
       </c>
       <c r="E93" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
       <c r="F93" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
       <c r="H93" s="1" t="s">
-        <v>238</v>
+        <v>192</v>
       </c>
     </row>
     <row r="94" spans="2:8">
       <c r="C94" s="1" t="s">
-        <v>239</v>
+        <v>193</v>
       </c>
       <c r="D94" s="1" t="s">
-        <v>192</v>
+        <v>146</v>
       </c>
       <c r="H94" s="1" t="s">
-        <v>234</v>
+        <v>188</v>
       </c>
     </row>
     <row r="95" spans="2:8">
       <c r="C95" s="1" t="s">
-        <v>240</v>
+        <v>194</v>
       </c>
       <c r="D95" s="1" t="s">
-        <v>192</v>
+        <v>146</v>
       </c>
       <c r="H95" s="1" t="s">
-        <v>235</v>
+        <v>189</v>
       </c>
     </row>
     <row r="96" spans="2:8">
       <c r="C96" s="1" t="s">
-        <v>303</v>
+        <v>256</v>
       </c>
       <c r="D96" s="1" t="s">
-        <v>228</v>
+        <v>268</v>
       </c>
     </row>
     <row r="97" spans="2:8">
       <c r="C97" s="1" t="s">
-        <v>304</v>
+        <v>257</v>
       </c>
       <c r="D97" s="1" t="s">
-        <v>159</v>
+        <v>113</v>
       </c>
     </row>
     <row r="100" spans="2:8">
       <c r="B100" s="1">
         <v>9</v>
       </c>
-      <c r="C100" s="21" t="s">
-        <v>197</v>
-      </c>
-      <c r="D100" s="21" t="s">
-        <v>193</v>
-      </c>
-      <c r="E100" s="21"/>
-      <c r="F100" s="21"/>
-      <c r="G100" s="21"/>
-      <c r="H100" s="21"/>
+      <c r="C100" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="D100" s="9" t="s">
+        <v>147</v>
+      </c>
+      <c r="E100" s="9"/>
+      <c r="F100" s="9"/>
+      <c r="G100" s="9"/>
+      <c r="H100" s="9"/>
     </row>
     <row r="101" spans="2:8">
       <c r="C101" s="7" t="s">
-        <v>162</v>
+        <v>116</v>
       </c>
       <c r="D101" s="7" t="s">
-        <v>163</v>
+        <v>117</v>
       </c>
       <c r="E101" s="7" t="s">
-        <v>164</v>
+        <v>118</v>
       </c>
       <c r="F101" s="7" t="s">
-        <v>166</v>
+        <v>120</v>
       </c>
       <c r="G101" s="7" t="s">
-        <v>188</v>
+        <v>142</v>
       </c>
       <c r="H101" s="7" t="s">
-        <v>167</v>
+        <v>121</v>
       </c>
     </row>
     <row r="102" spans="2:8">
       <c r="C102" s="1" t="s">
-        <v>175</v>
+        <v>129</v>
       </c>
       <c r="D102" s="1" t="s">
-        <v>159</v>
+        <v>113</v>
       </c>
       <c r="E102" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
       <c r="F102" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
       <c r="G102" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
       <c r="H102" s="1" t="s">
-        <v>219</v>
+        <v>173</v>
       </c>
     </row>
     <row r="103" spans="2:8">
       <c r="C103" s="1" t="s">
-        <v>281</v>
+        <v>234</v>
       </c>
       <c r="D103" s="1" t="s">
-        <v>159</v>
+        <v>113</v>
       </c>
       <c r="E103" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="H103" s="1" t="s">
         <v>165</v>
-      </c>
-      <c r="H103" s="1" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="104" spans="2:8">
       <c r="C104" s="1" t="s">
-        <v>282</v>
+        <v>235</v>
       </c>
       <c r="D104" s="1" t="s">
-        <v>161</v>
+        <v>115</v>
       </c>
       <c r="E104" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
       <c r="H104" s="1" t="s">
-        <v>210</v>
+        <v>164</v>
       </c>
     </row>
     <row r="105" spans="2:8">
       <c r="C105" s="1" t="s">
-        <v>195</v>
+        <v>149</v>
       </c>
       <c r="D105" s="1" t="s">
-        <v>192</v>
+        <v>146</v>
       </c>
     </row>
     <row r="106" spans="2:8">
       <c r="C106" s="1" t="s">
-        <v>283</v>
+        <v>236</v>
       </c>
       <c r="D106" s="1" t="s">
-        <v>192</v>
+        <v>146</v>
       </c>
     </row>
     <row r="107" spans="2:8">
       <c r="C107" s="1" t="s">
-        <v>284</v>
+        <v>237</v>
       </c>
       <c r="D107" s="1" t="s">
-        <v>192</v>
+        <v>146</v>
       </c>
     </row>
     <row r="108" spans="2:8">
       <c r="C108" s="1" t="s">
-        <v>196</v>
+        <v>150</v>
       </c>
       <c r="D108" s="1" t="s">
-        <v>192</v>
+        <v>146</v>
       </c>
     </row>
     <row r="109" spans="2:8">
       <c r="C109" s="1" t="s">
-        <v>197</v>
+        <v>151</v>
       </c>
       <c r="D109" s="1" t="s">
-        <v>192</v>
+        <v>146</v>
       </c>
     </row>
     <row r="110" spans="2:8">
       <c r="C110" s="1" t="s">
-        <v>199</v>
+        <v>153</v>
       </c>
       <c r="D110" s="1" t="s">
-        <v>159</v>
+        <v>113</v>
       </c>
       <c r="F110" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
     </row>
     <row r="111" spans="2:8">
       <c r="C111" s="1" t="s">
-        <v>198</v>
+        <v>152</v>
       </c>
       <c r="D111" s="1" t="s">
-        <v>192</v>
+        <v>146</v>
       </c>
     </row>
     <row r="112" spans="2:8">
       <c r="C112" s="1" t="s">
-        <v>256</v>
+        <v>210</v>
       </c>
       <c r="D112" s="1" t="s">
-        <v>228</v>
+        <v>268</v>
       </c>
       <c r="G112" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
     </row>
     <row r="113" spans="2:8">
       <c r="C113" s="1" t="s">
-        <v>302</v>
+        <v>255</v>
       </c>
       <c r="D113" s="1" t="s">
-        <v>159</v>
+        <v>113</v>
       </c>
       <c r="G113" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
     </row>
     <row r="114" spans="2:8">
       <c r="C114" s="1" t="s">
-        <v>303</v>
+        <v>256</v>
       </c>
       <c r="D114" s="1" t="s">
-        <v>228</v>
+        <v>268</v>
       </c>
     </row>
     <row r="115" spans="2:8">
       <c r="C115" s="1" t="s">
-        <v>304</v>
+        <v>257</v>
       </c>
       <c r="D115" s="1" t="s">
-        <v>159</v>
+        <v>113</v>
       </c>
     </row>
     <row r="117" spans="2:8">
       <c r="B117" s="1">
         <v>10</v>
       </c>
-      <c r="C117" s="21" t="s">
-        <v>202</v>
-      </c>
-      <c r="D117" s="21" t="s">
-        <v>203</v>
-      </c>
-      <c r="E117" s="21"/>
-      <c r="F117" s="21"/>
-      <c r="G117" s="21"/>
-      <c r="H117" s="21"/>
+      <c r="C117" s="9" t="s">
+        <v>156</v>
+      </c>
+      <c r="D117" s="9" t="s">
+        <v>157</v>
+      </c>
+      <c r="E117" s="9"/>
+      <c r="F117" s="9"/>
+      <c r="G117" s="9"/>
+      <c r="H117" s="9"/>
     </row>
     <row r="118" spans="2:8">
       <c r="C118" s="7" t="s">
-        <v>162</v>
+        <v>116</v>
       </c>
       <c r="D118" s="7" t="s">
-        <v>163</v>
+        <v>117</v>
       </c>
       <c r="E118" s="7" t="s">
-        <v>164</v>
+        <v>118</v>
       </c>
       <c r="F118" s="7" t="s">
-        <v>166</v>
+        <v>120</v>
       </c>
       <c r="G118" s="7" t="s">
-        <v>188</v>
+        <v>142</v>
       </c>
       <c r="H118" s="7" t="s">
-        <v>167</v>
+        <v>121</v>
       </c>
     </row>
     <row r="119" spans="2:8">
       <c r="C119" s="1" t="s">
-        <v>175</v>
+        <v>129</v>
       </c>
       <c r="D119" s="1" t="s">
-        <v>159</v>
+        <v>113</v>
       </c>
       <c r="E119" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
       <c r="F119" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
       <c r="G119" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
       <c r="H119" s="1" t="s">
-        <v>219</v>
+        <v>173</v>
       </c>
     </row>
     <row r="120" spans="2:8">
       <c r="C120" s="1" t="s">
-        <v>281</v>
+        <v>234</v>
       </c>
       <c r="D120" s="1" t="s">
-        <v>159</v>
+        <v>113</v>
       </c>
       <c r="E120" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="H120" s="1" t="s">
         <v>165</v>
-      </c>
-      <c r="H120" s="1" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="121" spans="2:8">
       <c r="C121" s="1" t="s">
-        <v>207</v>
+        <v>161</v>
       </c>
       <c r="D121" s="1" t="s">
-        <v>228</v>
+        <v>182</v>
       </c>
       <c r="E121" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
       <c r="H121" s="1" t="s">
-        <v>224</v>
+        <v>178</v>
       </c>
     </row>
     <row r="122" spans="2:8">
       <c r="C122" s="1" t="s">
-        <v>208</v>
+        <v>162</v>
       </c>
       <c r="D122" s="1" t="s">
-        <v>192</v>
+        <v>146</v>
       </c>
       <c r="G122" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
       <c r="H122" s="1" t="s">
-        <v>225</v>
+        <v>179</v>
       </c>
     </row>
     <row r="123" spans="2:8">
       <c r="C123" s="1" t="s">
-        <v>227</v>
+        <v>181</v>
       </c>
       <c r="D123" s="1" t="s">
-        <v>192</v>
+        <v>146</v>
       </c>
       <c r="H123" s="1" t="s">
-        <v>226</v>
+        <v>180</v>
       </c>
     </row>
     <row r="124" spans="2:8">
       <c r="C124" s="1" t="s">
-        <v>229</v>
+        <v>183</v>
       </c>
       <c r="D124" s="1" t="s">
-        <v>228</v>
+        <v>182</v>
       </c>
       <c r="H124" s="1" t="s">
-        <v>230</v>
+        <v>184</v>
       </c>
     </row>
     <row r="125" spans="2:8">
       <c r="C125" s="1" t="s">
-        <v>232</v>
+        <v>186</v>
       </c>
       <c r="D125" s="1" t="s">
-        <v>159</v>
+        <v>113</v>
       </c>
       <c r="H125" s="1" t="s">
-        <v>231</v>
+        <v>185</v>
       </c>
     </row>
     <row r="126" spans="2:8">
       <c r="C126" s="1" t="s">
-        <v>256</v>
+        <v>210</v>
       </c>
       <c r="D126" s="1" t="s">
-        <v>228</v>
+        <v>268</v>
       </c>
       <c r="G126" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
     </row>
     <row r="127" spans="2:8">
       <c r="C127" s="1" t="s">
-        <v>302</v>
+        <v>255</v>
       </c>
       <c r="D127" s="1" t="s">
-        <v>159</v>
+        <v>113</v>
       </c>
       <c r="G127" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
     </row>
     <row r="128" spans="2:8">
       <c r="C128" s="1" t="s">
-        <v>303</v>
+        <v>256</v>
       </c>
       <c r="D128" s="1" t="s">
-        <v>228</v>
+        <v>268</v>
       </c>
     </row>
     <row r="129" spans="2:8">
       <c r="C129" s="1" t="s">
-        <v>304</v>
+        <v>257</v>
       </c>
       <c r="D129" s="1" t="s">
-        <v>159</v>
+        <v>113</v>
       </c>
     </row>
     <row r="131" spans="2:8">
       <c r="B131" s="1">
         <v>11</v>
       </c>
-      <c r="C131" s="21" t="s">
-        <v>309</v>
-      </c>
-      <c r="D131" s="21" t="s">
-        <v>308</v>
-      </c>
-      <c r="E131" s="21"/>
-      <c r="F131" s="21"/>
-      <c r="G131" s="21"/>
-      <c r="H131" s="21"/>
+      <c r="C131" s="9" t="s">
+        <v>262</v>
+      </c>
+      <c r="D131" s="9" t="s">
+        <v>261</v>
+      </c>
+      <c r="E131" s="9"/>
+      <c r="F131" s="9"/>
+      <c r="G131" s="9"/>
+      <c r="H131" s="9"/>
     </row>
     <row r="132" spans="2:8">
       <c r="C132" s="7" t="s">
-        <v>162</v>
+        <v>116</v>
       </c>
       <c r="D132" s="7" t="s">
-        <v>163</v>
+        <v>117</v>
       </c>
       <c r="E132" s="7" t="s">
-        <v>164</v>
+        <v>118</v>
       </c>
       <c r="F132" s="7" t="s">
-        <v>166</v>
+        <v>120</v>
       </c>
       <c r="G132" s="7" t="s">
-        <v>188</v>
+        <v>142</v>
       </c>
       <c r="H132" s="7" t="s">
-        <v>167</v>
+        <v>121</v>
+      </c>
+    </row>
+    <row r="133" spans="2:8">
+      <c r="C133" s="1" t="s">
+        <v>275</v>
+      </c>
+      <c r="D133" s="1" t="s">
+        <v>273</v>
+      </c>
+      <c r="E133" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="G133" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="H133" s="1" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="134" spans="2:8">
+      <c r="C134" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="D134" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="G134" s="1" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="135" spans="2:8">
       <c r="C135" s="1" t="s">
-        <v>256</v>
+        <v>270</v>
       </c>
       <c r="D135" s="1" t="s">
-        <v>228</v>
+        <v>135</v>
       </c>
       <c r="G135" s="1" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
     </row>
     <row r="136" spans="2:8">
       <c r="C136" s="1" t="s">
-        <v>302</v>
+        <v>271</v>
       </c>
       <c r="D136" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="G136" s="1" t="s">
-        <v>165</v>
+        <v>146</v>
+      </c>
+    </row>
+    <row r="137" spans="2:8">
+      <c r="C137" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="D137" s="1" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="138" spans="2:8">
+      <c r="C138" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="D138" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="H138" s="1" t="s">
+        <v>276</v>
       </c>
     </row>
   </sheetData>
@@ -7472,317 +6614,317 @@
       <c r="B2" s="1">
         <v>1</v>
       </c>
-      <c r="C2" s="21" t="s">
-        <v>241</v>
-      </c>
-      <c r="D2" s="21" t="s">
-        <v>243</v>
-      </c>
-      <c r="E2" s="21" t="s">
-        <v>242</v>
-      </c>
-      <c r="F2" s="21"/>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
+      <c r="C2" s="9" t="s">
+        <v>195</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>197</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>196</v>
+      </c>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
     </row>
     <row r="3" spans="2:8">
       <c r="C3" s="7" t="s">
-        <v>246</v>
+        <v>200</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>244</v>
+        <v>198</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>245</v>
+        <v>199</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>249</v>
+        <v>203</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>250</v>
+        <v>204</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>285</v>
+        <v>238</v>
       </c>
     </row>
     <row r="4" spans="2:8" ht="31.5">
       <c r="C4" s="1" t="s">
-        <v>247</v>
+        <v>201</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>248</v>
-      </c>
-      <c r="E4" s="22" t="s">
-        <v>251</v>
-      </c>
-      <c r="G4" s="22" t="s">
-        <v>254</v>
+        <v>202</v>
+      </c>
+      <c r="E4" s="10" t="s">
+        <v>205</v>
+      </c>
+      <c r="G4" s="10" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="5" spans="2:8">
       <c r="C5" s="1" t="s">
-        <v>204</v>
+        <v>158</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>252</v>
+        <v>206</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>205</v>
+        <v>159</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>253</v>
+        <v>207</v>
       </c>
     </row>
     <row r="6" spans="2:8">
       <c r="D6" s="1" t="s">
-        <v>260</v>
+        <v>214</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>205</v>
+        <v>159</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>255</v>
+        <v>209</v>
       </c>
     </row>
     <row r="7" spans="2:8">
       <c r="C7" s="1" t="s">
-        <v>262</v>
+        <v>216</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>272</v>
+        <v>226</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>261</v>
+        <v>215</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>253</v>
+        <v>207</v>
       </c>
     </row>
     <row r="8" spans="2:8">
       <c r="D8" s="1" t="s">
-        <v>273</v>
+        <v>227</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>261</v>
+        <v>215</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>255</v>
+        <v>209</v>
       </c>
     </row>
     <row r="9" spans="2:8">
       <c r="C9" s="1" t="s">
-        <v>268</v>
+        <v>222</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>271</v>
+        <v>225</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>270</v>
+        <v>224</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>253</v>
+        <v>207</v>
       </c>
     </row>
     <row r="10" spans="2:8">
       <c r="D10" s="1" t="s">
-        <v>271</v>
+        <v>225</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>269</v>
+        <v>223</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>255</v>
+        <v>209</v>
       </c>
     </row>
     <row r="11" spans="2:8">
       <c r="C11" s="1" t="s">
-        <v>258</v>
+        <v>212</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>259</v>
+        <v>213</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>174</v>
+        <v>128</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>253</v>
+        <v>207</v>
       </c>
     </row>
     <row r="12" spans="2:8">
       <c r="D12" s="1" t="s">
-        <v>259</v>
+        <v>213</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>174</v>
+        <v>128</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>255</v>
+        <v>209</v>
       </c>
     </row>
     <row r="19" spans="2:8">
       <c r="B19" s="1">
         <v>2</v>
       </c>
-      <c r="C19" s="21" t="s">
-        <v>241</v>
-      </c>
-      <c r="D19" s="21" t="s">
-        <v>243</v>
-      </c>
-      <c r="E19" s="21" t="s">
-        <v>242</v>
-      </c>
-      <c r="F19" s="21"/>
-      <c r="G19" s="21"/>
-      <c r="H19" s="21"/>
+      <c r="C19" s="9" t="s">
+        <v>195</v>
+      </c>
+      <c r="D19" s="9" t="s">
+        <v>197</v>
+      </c>
+      <c r="E19" s="9" t="s">
+        <v>196</v>
+      </c>
+      <c r="F19" s="9"/>
+      <c r="G19" s="9"/>
+      <c r="H19" s="9"/>
     </row>
     <row r="20" spans="2:8">
       <c r="C20" s="7" t="s">
-        <v>246</v>
+        <v>200</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>244</v>
+        <v>198</v>
       </c>
       <c r="E20" s="7" t="s">
-        <v>245</v>
+        <v>199</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>249</v>
+        <v>203</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>250</v>
+        <v>204</v>
       </c>
       <c r="H20" s="7" t="s">
-        <v>285</v>
+        <v>238</v>
       </c>
     </row>
     <row r="21" spans="2:8">
       <c r="C21" s="1" t="s">
-        <v>274</v>
+        <v>228</v>
       </c>
     </row>
     <row r="22" spans="2:8">
       <c r="C22" s="1" t="s">
-        <v>287</v>
+        <v>240</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>286</v>
+        <v>239</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>290</v>
+        <v>243</v>
       </c>
     </row>
     <row r="23" spans="2:8">
       <c r="D23" s="1" t="s">
-        <v>275</v>
+        <v>229</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>290</v>
+        <v>243</v>
       </c>
     </row>
     <row r="27" spans="2:8">
-      <c r="C27" s="21" t="s">
-        <v>241</v>
-      </c>
-      <c r="D27" s="21" t="s">
-        <v>243</v>
-      </c>
-      <c r="E27" s="21" t="s">
-        <v>242</v>
-      </c>
-      <c r="F27" s="21"/>
-      <c r="G27" s="21"/>
-      <c r="H27" s="21"/>
+      <c r="C27" s="9" t="s">
+        <v>195</v>
+      </c>
+      <c r="D27" s="9" t="s">
+        <v>197</v>
+      </c>
+      <c r="E27" s="9" t="s">
+        <v>196</v>
+      </c>
+      <c r="F27" s="9"/>
+      <c r="G27" s="9"/>
+      <c r="H27" s="9"/>
     </row>
     <row r="28" spans="2:8">
       <c r="C28" s="7" t="s">
-        <v>246</v>
+        <v>200</v>
       </c>
       <c r="D28" s="7" t="s">
-        <v>244</v>
+        <v>198</v>
       </c>
       <c r="E28" s="7" t="s">
-        <v>245</v>
+        <v>199</v>
       </c>
       <c r="F28" s="7" t="s">
-        <v>249</v>
+        <v>203</v>
       </c>
       <c r="G28" s="7" t="s">
-        <v>250</v>
+        <v>204</v>
       </c>
       <c r="H28" s="7"/>
     </row>
     <row r="29" spans="2:8">
       <c r="C29" s="1" t="s">
-        <v>274</v>
+        <v>228</v>
       </c>
     </row>
     <row r="30" spans="2:8">
       <c r="C30" s="1" t="s">
-        <v>288</v>
+        <v>241</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>289</v>
+        <v>242</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>290</v>
+        <v>243</v>
       </c>
     </row>
     <row r="31" spans="2:8">
       <c r="C31" s="1" t="s">
-        <v>291</v>
+        <v>244</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>275</v>
+        <v>229</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>290</v>
+        <v>243</v>
       </c>
     </row>
     <row r="34" spans="3:8">
-      <c r="C34" s="21" t="s">
-        <v>241</v>
-      </c>
-      <c r="D34" s="21" t="s">
-        <v>202</v>
-      </c>
-      <c r="E34" s="21" t="s">
-        <v>292</v>
-      </c>
-      <c r="F34" s="21"/>
-      <c r="G34" s="21"/>
-      <c r="H34" s="21"/>
+      <c r="C34" s="9" t="s">
+        <v>195</v>
+      </c>
+      <c r="D34" s="9" t="s">
+        <v>156</v>
+      </c>
+      <c r="E34" s="9" t="s">
+        <v>245</v>
+      </c>
+      <c r="F34" s="9"/>
+      <c r="G34" s="9"/>
+      <c r="H34" s="9"/>
     </row>
     <row r="35" spans="3:8">
       <c r="C35" s="7" t="s">
-        <v>246</v>
+        <v>200</v>
       </c>
       <c r="D35" s="7" t="s">
-        <v>244</v>
+        <v>198</v>
       </c>
       <c r="E35" s="7" t="s">
-        <v>245</v>
+        <v>199</v>
       </c>
       <c r="F35" s="7" t="s">
-        <v>249</v>
+        <v>203</v>
       </c>
       <c r="G35" s="7" t="s">
-        <v>250</v>
+        <v>204</v>
       </c>
       <c r="H35" s="7"/>
     </row>
     <row r="36" spans="3:8" ht="31.5">
       <c r="C36" s="1" t="s">
-        <v>247</v>
+        <v>201</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>248</v>
-      </c>
-      <c r="E36" s="22" t="s">
-        <v>251</v>
-      </c>
-      <c r="G36" s="22" t="s">
-        <v>254</v>
+        <v>202</v>
+      </c>
+      <c r="E36" s="10" t="s">
+        <v>205</v>
+      </c>
+      <c r="G36" s="10" t="s">
+        <v>208</v>
       </c>
     </row>
   </sheetData>
@@ -7800,119 +6942,119 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" s="6" customFormat="1">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="8" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="1" t="s">
-        <v>293</v>
+        <v>246</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="1" t="s">
-        <v>301</v>
+        <v>254</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="1" t="s">
-        <v>299</v>
+        <v>252</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>294</v>
+        <v>247</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="1" t="s">
-        <v>301</v>
+        <v>254</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="1" t="s">
-        <v>299</v>
+        <v>252</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>93</v>
+        <v>84</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" s="1" t="s">
-        <v>301</v>
+        <v>254</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>299</v>
+        <v>252</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>300</v>
+        <v>253</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" s="1" t="s">
-        <v>301</v>
+        <v>254</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" s="1" t="s">
-        <v>299</v>
+        <v>252</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>295</v>
+        <v>248</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" s="1" t="s">
-        <v>301</v>
+        <v>254</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>299</v>
+        <v>252</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>298</v>
+        <v>251</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" s="1" t="s">
-        <v>301</v>
+        <v>254</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>299</v>
+        <v>252</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>297</v>
+        <v>250</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" s="1" t="s">
-        <v>301</v>
+        <v>254</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" s="1" t="s">
-        <v>299</v>
+        <v>252</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>296</v>
+        <v>249</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="B14" s="1" t="s">
-        <v>299</v>
+        <v>252</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>298</v>
+        <v>251</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="B15" s="1" t="s">
-        <v>299</v>
+        <v>252</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>297</v>
+        <v>250</v>
       </c>
     </row>
     <row r="18" spans="1:1" s="7" customFormat="1">
       <c r="A18" s="7" t="s">
-        <v>310</v>
+        <v>263</v>
       </c>
     </row>
   </sheetData>
@@ -7932,20 +7074,20 @@
   <sheetData>
     <row r="1" spans="1:5" s="6" customFormat="1" ht="18.75">
       <c r="A1" s="6" t="s">
-        <v>311</v>
-      </c>
-      <c r="E1" s="24" t="s">
-        <v>312</v>
+        <v>264</v>
+      </c>
+      <c r="E1" s="12" t="s">
+        <v>265</v>
       </c>
     </row>
     <row r="34" spans="2:2">
       <c r="B34" s="1" t="s">
-        <v>313</v>
+        <v>266</v>
       </c>
     </row>
     <row r="83" spans="2:2">
       <c r="B83" s="1" t="s">
-        <v>314</v>
+        <v>267</v>
       </c>
     </row>
   </sheetData>
@@ -7959,581 +7101,16 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{954BCFCB-6BAA-41A6-B08B-38BC3239599E}">
-  <sheetPr>
-    <tabColor theme="0" tint="-0.499984740745262"/>
-  </sheetPr>
-  <dimension ref="A1:AI63"/>
-  <sheetFormatPr defaultColWidth="4.75" defaultRowHeight="15.75"/>
-  <cols>
-    <col min="1" max="16384" width="4.75" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:35" s="6" customFormat="1">
-      <c r="A1" s="18" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="2" spans="1:35" s="7" customFormat="1">
-      <c r="A2" s="17" t="s">
-        <v>84</v>
-      </c>
-      <c r="B2" s="8"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
-      <c r="H2" s="8"/>
-      <c r="I2" s="8"/>
-      <c r="J2" s="8"/>
-      <c r="K2" s="8"/>
-      <c r="L2" s="8"/>
-      <c r="M2" s="8"/>
-      <c r="N2" s="8"/>
-      <c r="O2" s="8"/>
-      <c r="P2" s="9"/>
-      <c r="Q2" s="17" t="s">
-        <v>94</v>
-      </c>
-      <c r="R2" s="8"/>
-      <c r="S2" s="8"/>
-      <c r="T2" s="8"/>
-      <c r="U2" s="8"/>
-      <c r="V2" s="8"/>
-      <c r="W2" s="8"/>
-      <c r="X2" s="8"/>
-      <c r="Y2" s="8"/>
-      <c r="Z2" s="8"/>
-      <c r="AA2" s="8"/>
-      <c r="AB2" s="8"/>
-      <c r="AC2" s="8"/>
-      <c r="AD2" s="8"/>
-      <c r="AE2" s="8"/>
-      <c r="AF2" s="8"/>
-      <c r="AG2" s="8"/>
-      <c r="AH2" s="8"/>
-      <c r="AI2" s="9"/>
-    </row>
-    <row r="3" spans="1:35">
-      <c r="A3" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="P3" s="11"/>
-      <c r="Q3" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="S3" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="AI3" s="11"/>
-    </row>
-    <row r="4" spans="1:35">
-      <c r="A4" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="P4" s="11"/>
-      <c r="Q4" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="R4" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="AA4" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="AI4" s="11"/>
-    </row>
-    <row r="5" spans="1:35">
-      <c r="A5" s="19"/>
-      <c r="B5" s="20" t="s">
-        <v>111</v>
-      </c>
-      <c r="P5" s="11"/>
-      <c r="Q5" s="19"/>
-      <c r="R5" s="20" t="s">
-        <v>111</v>
-      </c>
-      <c r="AI5" s="11"/>
-    </row>
-    <row r="6" spans="1:35">
-      <c r="A6" s="10"/>
-      <c r="B6" s="20" t="s">
-        <v>102</v>
-      </c>
-      <c r="P6" s="11"/>
-      <c r="Q6" s="10"/>
-      <c r="R6" s="20" t="s">
-        <v>112</v>
-      </c>
-      <c r="AI6" s="11"/>
-    </row>
-    <row r="7" spans="1:35">
-      <c r="A7" s="10"/>
-      <c r="B7" s="20" t="s">
-        <v>99</v>
-      </c>
-      <c r="P7" s="11"/>
-      <c r="Q7" s="10"/>
-      <c r="T7" s="20" t="s">
-        <v>113</v>
-      </c>
-      <c r="AI7" s="11"/>
-    </row>
-    <row r="8" spans="1:35">
-      <c r="A8" s="10"/>
-      <c r="B8" s="20" t="s">
-        <v>103</v>
-      </c>
-      <c r="P8" s="11"/>
-      <c r="Q8" s="10"/>
-      <c r="T8" s="20" t="s">
-        <v>122</v>
-      </c>
-      <c r="AI8" s="11"/>
-    </row>
-    <row r="9" spans="1:35">
-      <c r="A9" s="10"/>
-      <c r="P9" s="11"/>
-      <c r="Q9" s="10"/>
-      <c r="R9" s="20" t="s">
-        <v>107</v>
-      </c>
-      <c r="AI9" s="11"/>
-    </row>
-    <row r="10" spans="1:35">
-      <c r="A10" s="10"/>
-      <c r="P10" s="11"/>
-      <c r="Q10" s="10"/>
-      <c r="R10" s="20" t="s">
-        <v>108</v>
-      </c>
-      <c r="AI10" s="11"/>
-    </row>
-    <row r="11" spans="1:35">
-      <c r="P11" s="11"/>
-      <c r="R11" s="20" t="s">
-        <v>109</v>
-      </c>
-      <c r="AI11" s="11"/>
-    </row>
-    <row r="12" spans="1:35">
-      <c r="P12" s="11"/>
-      <c r="R12" s="20" t="s">
-        <v>110</v>
-      </c>
-      <c r="AI12" s="11"/>
-    </row>
-    <row r="13" spans="1:35">
-      <c r="A13" s="10"/>
-      <c r="P13" s="11"/>
-      <c r="Q13" s="10"/>
-      <c r="R13" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="AI13" s="11"/>
-    </row>
-    <row r="14" spans="1:35">
-      <c r="A14" s="10"/>
-      <c r="P14" s="11"/>
-      <c r="Q14" s="10"/>
-      <c r="AI14" s="11"/>
-    </row>
-    <row r="15" spans="1:35">
-      <c r="A15" s="10"/>
-      <c r="P15" s="11"/>
-      <c r="Q15" s="10"/>
-      <c r="AI15" s="11"/>
-    </row>
-    <row r="16" spans="1:35">
-      <c r="A16" s="15" t="s">
-        <v>85</v>
-      </c>
-      <c r="B16" s="16"/>
-      <c r="C16" s="16"/>
-      <c r="D16" s="16"/>
-      <c r="E16" s="16"/>
-      <c r="F16" s="16"/>
-      <c r="G16" s="16"/>
-      <c r="H16" s="16"/>
-      <c r="P16" s="11"/>
-      <c r="Q16" s="15" t="s">
-        <v>85</v>
-      </c>
-      <c r="R16" s="16"/>
-      <c r="S16" s="16"/>
-      <c r="T16" s="16"/>
-      <c r="U16" s="16"/>
-      <c r="V16" s="16"/>
-      <c r="W16" s="16"/>
-      <c r="X16" s="16"/>
-      <c r="Y16" s="16"/>
-      <c r="Z16" s="16"/>
-      <c r="AA16" s="16"/>
-      <c r="AI16" s="11"/>
-    </row>
-    <row r="17" spans="1:35">
-      <c r="A17" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="B17" s="16"/>
-      <c r="C17" s="16"/>
-      <c r="D17" s="16"/>
-      <c r="E17" s="16"/>
-      <c r="F17" s="16"/>
-      <c r="G17" s="16"/>
-      <c r="H17" s="16"/>
-      <c r="P17" s="11"/>
-      <c r="Q17" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="R17" s="16"/>
-      <c r="S17" s="16"/>
-      <c r="T17" s="16"/>
-      <c r="U17" s="16"/>
-      <c r="V17" s="16"/>
-      <c r="W17" s="16"/>
-      <c r="X17" s="16"/>
-      <c r="Y17" s="16"/>
-      <c r="Z17" s="16"/>
-      <c r="AA17" s="16"/>
-      <c r="AI17" s="11"/>
-    </row>
-    <row r="18" spans="1:35">
-      <c r="A18" s="15" t="s">
-        <v>91</v>
-      </c>
-      <c r="B18" s="16" t="s">
-        <v>106</v>
-      </c>
-      <c r="C18" s="16"/>
-      <c r="D18" s="16"/>
-      <c r="E18" s="16"/>
-      <c r="F18" s="16"/>
-      <c r="G18" s="16"/>
-      <c r="H18" s="16"/>
-      <c r="P18" s="11"/>
-      <c r="Q18" s="15" t="s">
-        <v>91</v>
-      </c>
-      <c r="R18" s="16" t="s">
-        <v>105</v>
-      </c>
-      <c r="S18" s="16"/>
-      <c r="T18" s="16"/>
-      <c r="U18" s="16"/>
-      <c r="V18" s="16"/>
-      <c r="W18" s="16"/>
-      <c r="X18" s="16"/>
-      <c r="Y18" s="16"/>
-      <c r="Z18" s="16"/>
-      <c r="AA18" s="16"/>
-      <c r="AI18" s="11"/>
-    </row>
-    <row r="19" spans="1:35">
-      <c r="A19" s="15"/>
-      <c r="B19" s="16"/>
-      <c r="C19" s="16"/>
-      <c r="D19" s="16"/>
-      <c r="E19" s="16"/>
-      <c r="F19" s="16"/>
-      <c r="G19" s="16"/>
-      <c r="H19" s="16"/>
-      <c r="P19" s="11"/>
-      <c r="Q19" s="15"/>
-      <c r="R19" s="16"/>
-      <c r="S19" s="16"/>
-      <c r="T19" s="16"/>
-      <c r="U19" s="16"/>
-      <c r="V19" s="16"/>
-      <c r="W19" s="16"/>
-      <c r="X19" s="16"/>
-      <c r="Y19" s="16"/>
-      <c r="Z19" s="16"/>
-      <c r="AA19" s="16"/>
-      <c r="AI19" s="11"/>
-    </row>
-    <row r="20" spans="1:35">
-      <c r="A20" s="10" t="s">
-        <v>95</v>
-      </c>
-      <c r="P20" s="11"/>
-      <c r="Q20" s="10" t="s">
-        <v>95</v>
-      </c>
-      <c r="AI20" s="11"/>
-    </row>
-    <row r="21" spans="1:35">
-      <c r="A21" s="10" t="s">
-        <v>96</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="P21" s="11"/>
-      <c r="Q21" s="10" t="s">
-        <v>96</v>
-      </c>
-      <c r="S21" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="AI21" s="11"/>
-    </row>
-    <row r="22" spans="1:35">
-      <c r="A22" s="10"/>
-      <c r="P22" s="11"/>
-      <c r="Q22" s="10"/>
-      <c r="AI22" s="11"/>
-    </row>
-    <row r="23" spans="1:35">
-      <c r="A23" s="12"/>
-      <c r="B23" s="13"/>
-      <c r="C23" s="13"/>
-      <c r="D23" s="13"/>
-      <c r="E23" s="13"/>
-      <c r="F23" s="13"/>
-      <c r="G23" s="13"/>
-      <c r="H23" s="13"/>
-      <c r="I23" s="13"/>
-      <c r="J23" s="13"/>
-      <c r="K23" s="13"/>
-      <c r="L23" s="13"/>
-      <c r="M23" s="13"/>
-      <c r="N23" s="13"/>
-      <c r="O23" s="13"/>
-      <c r="P23" s="14"/>
-      <c r="Q23" s="12"/>
-      <c r="R23" s="13"/>
-      <c r="S23" s="13"/>
-      <c r="T23" s="13"/>
-      <c r="U23" s="13"/>
-      <c r="V23" s="13"/>
-      <c r="W23" s="13"/>
-      <c r="X23" s="13"/>
-      <c r="Y23" s="13"/>
-      <c r="Z23" s="13"/>
-      <c r="AA23" s="13"/>
-      <c r="AB23" s="13"/>
-      <c r="AC23" s="13"/>
-      <c r="AD23" s="13"/>
-      <c r="AE23" s="13"/>
-      <c r="AF23" s="13"/>
-      <c r="AG23" s="13"/>
-      <c r="AH23" s="13"/>
-      <c r="AI23" s="14"/>
-    </row>
-    <row r="24" spans="1:35">
-      <c r="A24" s="17" t="s">
-        <v>90</v>
-      </c>
-      <c r="B24" s="8"/>
-      <c r="C24" s="8" t="s">
-        <v>88</v>
-      </c>
-      <c r="D24" s="8"/>
-      <c r="E24" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="F24" s="8"/>
-      <c r="G24" s="8"/>
-      <c r="H24" s="8"/>
-      <c r="I24" s="8"/>
-      <c r="J24" s="8"/>
-      <c r="K24" s="8"/>
-      <c r="L24" s="8"/>
-      <c r="M24" s="8"/>
-      <c r="N24" s="8"/>
-      <c r="O24" s="8"/>
-      <c r="P24" s="8"/>
-      <c r="Q24" s="8"/>
-      <c r="R24" s="8"/>
-      <c r="S24" s="8"/>
-      <c r="T24" s="8"/>
-      <c r="U24" s="8"/>
-      <c r="V24" s="8"/>
-      <c r="W24" s="8"/>
-      <c r="X24" s="8"/>
-      <c r="Y24" s="8"/>
-      <c r="Z24" s="8"/>
-      <c r="AA24" s="8"/>
-      <c r="AB24" s="8"/>
-      <c r="AC24" s="8"/>
-      <c r="AD24" s="8"/>
-      <c r="AE24" s="8"/>
-      <c r="AF24" s="8"/>
-      <c r="AG24" s="8"/>
-      <c r="AH24" s="8"/>
-      <c r="AI24" s="9"/>
-    </row>
-    <row r="25" spans="1:35">
-      <c r="A25" s="10" t="s">
-        <v>91</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="AI25" s="11"/>
-    </row>
-    <row r="26" spans="1:35">
-      <c r="A26" s="12"/>
-      <c r="B26" s="13"/>
-      <c r="C26" s="13"/>
-      <c r="D26" s="13"/>
-      <c r="E26" s="13"/>
-      <c r="F26" s="13"/>
-      <c r="G26" s="13"/>
-      <c r="H26" s="13"/>
-      <c r="I26" s="13"/>
-      <c r="J26" s="13"/>
-      <c r="K26" s="13"/>
-      <c r="L26" s="13"/>
-      <c r="M26" s="13"/>
-      <c r="N26" s="13"/>
-      <c r="O26" s="13"/>
-      <c r="P26" s="13"/>
-      <c r="Q26" s="13"/>
-      <c r="R26" s="13"/>
-      <c r="S26" s="13"/>
-      <c r="T26" s="13"/>
-      <c r="U26" s="13"/>
-      <c r="V26" s="13"/>
-      <c r="W26" s="13"/>
-      <c r="X26" s="13"/>
-      <c r="Y26" s="13"/>
-      <c r="Z26" s="13"/>
-      <c r="AA26" s="13"/>
-      <c r="AB26" s="13"/>
-      <c r="AC26" s="13"/>
-      <c r="AD26" s="13"/>
-      <c r="AE26" s="13"/>
-      <c r="AF26" s="13"/>
-      <c r="AG26" s="13"/>
-      <c r="AH26" s="13"/>
-      <c r="AI26" s="14"/>
-    </row>
-    <row r="29" spans="1:35">
-      <c r="Q29" s="1" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="30" spans="1:35">
-      <c r="Q30" s="1" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="31" spans="1:35">
-      <c r="R31" s="1" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="35" spans="17:18">
-      <c r="Q35" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="36" spans="17:18">
-      <c r="R36" s="1" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="37" spans="17:18">
-      <c r="R37" s="1" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="52" spans="17:17">
-      <c r="Q52" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="63" spans="17:17">
-      <c r="Q63" s="1" t="s">
-        <v>121</v>
-      </c>
-    </row>
-  </sheetData>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E0CD117-9164-4B42-8B44-5B255580D7A3}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
+  <sheetData/>
   <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{264C402C-30BF-413A-B2A5-65201BF6F05B}">
-  <dimension ref="A1:J23"/>
-  <sheetFormatPr defaultColWidth="8.75" defaultRowHeight="15.75"/>
-  <cols>
-    <col min="1" max="16384" width="8.75" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:10" s="6" customFormat="1">
-      <c r="A1" s="7" t="s">
-        <v>124</v>
-      </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="H1" s="7"/>
-      <c r="I1" s="7"/>
-      <c r="J1" s="7"/>
-    </row>
-    <row r="2" spans="1:10">
-      <c r="A2" s="1" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10">
-      <c r="A3" s="1" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10">
-      <c r="A5" s="1" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10">
-      <c r="A6" s="1" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1">
-      <c r="A20" s="1" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1">
-      <c r="A21" s="1" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1">
-      <c r="A22" s="1" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1">
-      <c r="A23" s="1" t="s">
-        <v>131</v>
-      </c>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="1"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5394D207-6464-436E-ADE4-2A4026304978}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultColWidth="8.75" defaultRowHeight="15.75"/>
@@ -8547,7 +7124,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7C229AB-5092-49C9-8D15-67A2BD891095}">
   <dimension ref="A1:A77"/>
   <sheetFormatPr defaultColWidth="8.75" defaultRowHeight="15.75"/>
@@ -8672,4 +7249,209 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E00EB3AB-A229-45B6-BAF0-CBFC690801AC}">
+  <dimension ref="A1:A72"/>
+  <sheetFormatPr defaultColWidth="8.75" defaultRowHeight="15.75"/>
+  <cols>
+    <col min="1" max="16384" width="8.75" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" s="6" customFormat="1">
+      <c r="A1" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" s="7" customFormat="1">
+      <c r="A2" s="7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1">
+      <c r="A3" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1">
+      <c r="A5" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1">
+      <c r="A7" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1">
+      <c r="A8" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1">
+      <c r="A10" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1">
+      <c r="A11" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1">
+      <c r="A13" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1">
+      <c r="A14" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1">
+      <c r="A16" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1">
+      <c r="A17" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" s="7" customFormat="1">
+      <c r="A22" s="7" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1">
+      <c r="A23" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" s="7" customFormat="1">
+      <c r="A37" s="7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1">
+      <c r="A38" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1">
+      <c r="A40" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1">
+      <c r="A41" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1">
+      <c r="A43" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1">
+      <c r="A44" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1">
+      <c r="A45" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1">
+      <c r="A47" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1">
+      <c r="A48" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1">
+      <c r="A50" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1">
+      <c r="A51" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1">
+      <c r="A54" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1">
+      <c r="A55" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1">
+      <c r="A56" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1">
+      <c r="A57" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" s="7" customFormat="1">
+      <c r="A60" s="7" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1">
+      <c r="A62" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1">
+      <c r="A63" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1">
+      <c r="A65" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1">
+      <c r="A66" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1">
+      <c r="A68" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1">
+      <c r="A69" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1">
+      <c r="A71" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1">
+      <c r="A72" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>